<commit_message>
added spare parts inventory - basic
</commit_message>
<xml_diff>
--- a/vehicle renewal tracker.xlsx
+++ b/vehicle renewal tracker.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30015"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F50A8840-ED90-456B-BBB5-1F4F70E95F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E9AE5BD-0E41-4163-92A6-71990C3E43DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="renewal tracker" sheetId="1" r:id="rId1"/>
     <sheet name="maintenance log" sheetId="2" r:id="rId2"/>
+    <sheet name="spare parts" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="334">
   <si>
     <t>VEHICLE RENWAL TRACKER 2026 (BASIC)</t>
   </si>
@@ -659,6 +660,381 @@
   </si>
   <si>
     <t>Performance issue</t>
+  </si>
+  <si>
+    <t>SPARE PARTS INVENTORY - BASIC</t>
+  </si>
+  <si>
+    <t>Part Details</t>
+  </si>
+  <si>
+    <t>Supplier Details</t>
+  </si>
+  <si>
+    <t>Inventory Info</t>
+  </si>
+  <si>
+    <t>Part No.</t>
+  </si>
+  <si>
+    <t>Part Description</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Supplier Info</t>
+  </si>
+  <si>
+    <t>Contact</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Min. Stock</t>
+  </si>
+  <si>
+    <t>Balance</t>
+  </si>
+  <si>
+    <t>Last Restocked On</t>
+  </si>
+  <si>
+    <t>P-2001</t>
+  </si>
+  <si>
+    <t>Engine Oil 5W30</t>
+  </si>
+  <si>
+    <t>Lubricant</t>
+  </si>
+  <si>
+    <t>Shell</t>
+  </si>
+  <si>
+    <t>Shell Distributor</t>
+  </si>
+  <si>
+    <t>shell@fuel.com</t>
+  </si>
+  <si>
+    <t>Warehouse A</t>
+  </si>
+  <si>
+    <t>Shelf 1</t>
+  </si>
+  <si>
+    <t>Daily servicing</t>
+  </si>
+  <si>
+    <t>P-2002</t>
+  </si>
+  <si>
+    <t>Coolant</t>
+  </si>
+  <si>
+    <t>Gulf</t>
+  </si>
+  <si>
+    <t>Gulf Supplier</t>
+  </si>
+  <si>
+    <t>gulf@dealer.com</t>
+  </si>
+  <si>
+    <t>Shelf 2</t>
+  </si>
+  <si>
+    <t>Top-up usage</t>
+  </si>
+  <si>
+    <t>P-2003</t>
+  </si>
+  <si>
+    <t>Brake Fluid</t>
+  </si>
+  <si>
+    <t>Consumable</t>
+  </si>
+  <si>
+    <t>Bosch</t>
+  </si>
+  <si>
+    <t>Bosch Dealer</t>
+  </si>
+  <si>
+    <t>bosch@dealer.com</t>
+  </si>
+  <si>
+    <t>Shelf 3</t>
+  </si>
+  <si>
+    <t>Brake maintenance</t>
+  </si>
+  <si>
+    <t>P-2004</t>
+  </si>
+  <si>
+    <t>Wiper Blade Set</t>
+  </si>
+  <si>
+    <t>Spare Part</t>
+  </si>
+  <si>
+    <t>Bosch Supplier</t>
+  </si>
+  <si>
+    <t>bosch@parts.com</t>
+  </si>
+  <si>
+    <t>Warehouse B</t>
+  </si>
+  <si>
+    <t>Shelf 4</t>
+  </si>
+  <si>
+    <t>Replacement</t>
+  </si>
+  <si>
+    <t>P-2005</t>
+  </si>
+  <si>
+    <t>Mudflap Set</t>
+  </si>
+  <si>
+    <t>Body Part</t>
+  </si>
+  <si>
+    <t>Tata Dealer</t>
+  </si>
+  <si>
+    <t>tata@dealer.com</t>
+  </si>
+  <si>
+    <t>Shelf 5</t>
+  </si>
+  <si>
+    <t>Damaged replacement</t>
+  </si>
+  <si>
+    <t>P-2006</t>
+  </si>
+  <si>
+    <t>AdBlue (DEF)</t>
+  </si>
+  <si>
+    <t>Yard</t>
+  </si>
+  <si>
+    <t>Tank Storage</t>
+  </si>
+  <si>
+    <t>Daily usage</t>
+  </si>
+  <si>
+    <t>P-2007</t>
+  </si>
+  <si>
+    <t>Gear Oil</t>
+  </si>
+  <si>
+    <t>Castrol</t>
+  </si>
+  <si>
+    <t>Castrol Supplier</t>
+  </si>
+  <si>
+    <t>castrol@oil.com</t>
+  </si>
+  <si>
+    <t>Shelf 6</t>
+  </si>
+  <si>
+    <t>Gear top-up</t>
+  </si>
+  <si>
+    <t>P-2008</t>
+  </si>
+  <si>
+    <t>Differential Oil</t>
+  </si>
+  <si>
+    <t>Mobil</t>
+  </si>
+  <si>
+    <t>Mobil Dealer</t>
+  </si>
+  <si>
+    <t>mobil@oil.com</t>
+  </si>
+  <si>
+    <t>Shelf 7</t>
+  </si>
+  <si>
+    <t>Differential top-up</t>
+  </si>
+  <si>
+    <t>P-2009</t>
+  </si>
+  <si>
+    <t>Windshield Washer Fluid</t>
+  </si>
+  <si>
+    <t>3M</t>
+  </si>
+  <si>
+    <t>3M Supplier</t>
+  </si>
+  <si>
+    <t>3m@care.com</t>
+  </si>
+  <si>
+    <t>Shelf 8</t>
+  </si>
+  <si>
+    <t>Daily refill</t>
+  </si>
+  <si>
+    <t>P-2010</t>
+  </si>
+  <si>
+    <t>LED Headlight Bulb</t>
+  </si>
+  <si>
+    <t>Electrical</t>
+  </si>
+  <si>
+    <t>Philips</t>
+  </si>
+  <si>
+    <t>Philips Dealer</t>
+  </si>
+  <si>
+    <t>philips@lights.com</t>
+  </si>
+  <si>
+    <t>Shelf 9</t>
+  </si>
+  <si>
+    <t>P-2011</t>
+  </si>
+  <si>
+    <t>Indicator Bulb</t>
+  </si>
+  <si>
+    <t>Osram</t>
+  </si>
+  <si>
+    <t>Osram Supplier</t>
+  </si>
+  <si>
+    <t>osram@lights.com</t>
+  </si>
+  <si>
+    <t>Shelf 10</t>
+  </si>
+  <si>
+    <t>P-2012</t>
+  </si>
+  <si>
+    <t>Tail Light Bulb</t>
+  </si>
+  <si>
+    <t>Shelf 11</t>
+  </si>
+  <si>
+    <t>P-2013</t>
+  </si>
+  <si>
+    <t>Fuse Kit</t>
+  </si>
+  <si>
+    <t>Workshop</t>
+  </si>
+  <si>
+    <t>Tool Rack</t>
+  </si>
+  <si>
+    <t>Electrical fixes</t>
+  </si>
+  <si>
+    <t>P-2014</t>
+  </si>
+  <si>
+    <t>Cable Ties Pack</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Local Vendor</t>
+  </si>
+  <si>
+    <t>local@garage.com</t>
+  </si>
+  <si>
+    <t>Minor fixes</t>
+  </si>
+  <si>
+    <t>P-2015</t>
+  </si>
+  <si>
+    <t>Electrical Tape</t>
+  </si>
+  <si>
+    <t>Wiring repairs</t>
+  </si>
+  <si>
+    <t>P-2016</t>
+  </si>
+  <si>
+    <t>Grease</t>
+  </si>
+  <si>
+    <t>Shelf 12</t>
+  </si>
+  <si>
+    <t>Lubrication</t>
+  </si>
+  <si>
+    <t>P-2017</t>
+  </si>
+  <si>
+    <t>Microfiber Cloth</t>
+  </si>
+  <si>
+    <t>Cleaning Supplier</t>
+  </si>
+  <si>
+    <t>clean@supplies.com</t>
+  </si>
+  <si>
+    <t>Storage Rack</t>
+  </si>
+  <si>
+    <t>Cleaning</t>
+  </si>
+  <si>
+    <t>P-2018</t>
+  </si>
+  <si>
+    <t>Air Valve Cap</t>
+  </si>
+  <si>
+    <t>Small Part</t>
+  </si>
+  <si>
+    <t>Generic</t>
+  </si>
+  <si>
+    <t>local@parts.com</t>
+  </si>
+  <si>
+    <t>Shelf 13</t>
   </si>
 </sst>
 </file>
@@ -669,7 +1045,7 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
     <numFmt numFmtId="165" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -708,8 +1084,22 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="48"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -764,8 +1154,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="30">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -1162,11 +1570,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1252,33 +1691,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1311,12 +1723,555 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="34">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="20" formatCode="d\-mmm\-yy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -1363,6 +2318,64 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{285E3A23-AB6B-40AF-AAF2-8F052F572429}" name="Table3" displayName="Table3" ref="G5:J23" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26" headerRowBorderDxfId="24" tableBorderDxfId="25" totalsRowBorderDxfId="23">
+  <autoFilter ref="G5:J23" xr:uid="{285E3A23-AB6B-40AF-AAF2-8F052F572429}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{6F2BA377-D0DA-4E5B-946E-005591BD7895}" name="Supplier Info" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{763F2F7B-DC8A-4D33-AE92-8D462C1AF93B}" name="Contact" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{48307B2D-7A93-41FA-91BD-58DC279B1F52}" name="Email" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{11DEC9B0-4188-4D4D-978C-A993E46788B5}" name="Location" dataDxfId="19"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1A0D7FA3-B21E-4C9D-A9BC-12FE77589BA8}" name="Table5" displayName="Table5" ref="B5:F23" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17" headerRowBorderDxfId="15" tableBorderDxfId="16" totalsRowBorderDxfId="14">
+  <autoFilter ref="B5:F23" xr:uid="{1A0D7FA3-B21E-4C9D-A9BC-12FE77589BA8}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{37ACE421-A565-47AE-A2B6-A8A255E415C1}" name="SL.NO." dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{46CE06A5-F016-4BA1-82A3-6D69BA2ED96A}" name="Part No." dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{10306DC6-1168-455A-A8E8-481DE09EA2A4}" name="Part Description" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{495DEC6F-C09E-4FD1-8BD6-99A0B818D76E}" name="Category" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{DEC7BBDF-F80C-4103-8059-27FC043BF965}" name="Brand" dataDxfId="9"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{343224D2-3FDB-450A-B8BB-DCD1C7AF8D83}" name="Table6" displayName="Table6" ref="K5:O23" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+  <autoFilter ref="K5:O23" xr:uid="{343224D2-3FDB-450A-B8BB-DCD1C7AF8D83}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{D4F2BAB3-028C-42F2-A5B8-803EAC729AA1}" name="Min. Stock" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{EE24FA7D-5A52-496C-A701-9DCADF04EA0A}" name="Balance" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{128B8679-EF11-4250-9B8E-A3C459C212D7}" name="Location" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{8ECD204C-FC50-4A41-B1C9-E099E0846772}" name="Last Restocked On" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{486C6924-252C-460E-A9B2-63D11264BCA3}" name="Remarks" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1678,51 +2691,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:15">
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="33"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="44"/>
     </row>
     <row r="2" spans="3:15">
-      <c r="C2" s="34"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="35"/>
-      <c r="O2" s="36"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="46"/>
+      <c r="L2" s="46"/>
+      <c r="M2" s="46"/>
+      <c r="N2" s="46"/>
+      <c r="O2" s="47"/>
     </row>
     <row r="3" spans="3:15">
-      <c r="C3" s="37"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="38"/>
-      <c r="J3" s="38"/>
-      <c r="K3" s="38"/>
-      <c r="L3" s="38"/>
-      <c r="M3" s="38"/>
-      <c r="N3" s="38"/>
-      <c r="O3" s="39"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="49"/>
+      <c r="L3" s="49"/>
+      <c r="M3" s="49"/>
+      <c r="N3" s="49"/>
+      <c r="O3" s="50"/>
     </row>
     <row r="4" spans="3:15">
       <c r="C4" s="5" t="s">
@@ -2529,17 +3542,17 @@
     <mergeCell ref="C1:O3"/>
   </mergeCells>
   <conditionalFormatting sqref="O5:O22">
-    <cfRule type="cellIs" dxfId="2" priority="3" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="33" priority="3" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O5:O22">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="32" priority="2" operator="lessThanOrEqual">
       <formula>30</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O5:O22">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="31" priority="1" operator="between">
       <formula>31</formula>
       <formula>89</formula>
     </cfRule>
@@ -2568,72 +3581,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14">
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="39" t="s">
         <v>135</v>
       </c>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="49"/>
-      <c r="M1" s="49"/>
-      <c r="N1" s="49"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
     </row>
     <row r="2" spans="2:14">
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="49"/>
-      <c r="M2" s="49"/>
-      <c r="N2" s="49"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
+      <c r="K2" s="40"/>
+      <c r="L2" s="40"/>
+      <c r="M2" s="40"/>
+      <c r="N2" s="40"/>
     </row>
     <row r="3" spans="2:14">
-      <c r="B3" s="49"/>
-      <c r="C3" s="49"/>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="49"/>
-      <c r="H3" s="49"/>
-      <c r="I3" s="49"/>
-      <c r="J3" s="49"/>
-      <c r="K3" s="49"/>
-      <c r="L3" s="49"/>
-      <c r="M3" s="49"/>
-      <c r="N3" s="49"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+      <c r="K3" s="40"/>
+      <c r="L3" s="40"/>
+      <c r="M3" s="40"/>
+      <c r="N3" s="40"/>
     </row>
     <row r="4" spans="2:14">
-      <c r="B4" s="50"/>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
-      <c r="J4" s="50"/>
-      <c r="K4" s="50"/>
-      <c r="L4" s="50"/>
-      <c r="M4" s="50"/>
-      <c r="N4" s="50"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
+      <c r="M4" s="41"/>
+      <c r="N4" s="41"/>
     </row>
     <row r="5" spans="2:14">
       <c r="B5" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="C5" s="41" t="s">
+      <c r="C5" s="32" t="s">
         <v>137</v>
       </c>
       <c r="D5" s="17" t="s">
@@ -2674,37 +3687,37 @@
       <c r="B6" s="1">
         <v>1</v>
       </c>
-      <c r="C6" s="42">
+      <c r="C6" s="33">
         <v>46032</v>
       </c>
-      <c r="D6" s="43" t="s">
+      <c r="D6" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="43" t="s">
+      <c r="E6" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="44" t="s">
+      <c r="F6" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="44" t="s">
+      <c r="G6" s="35" t="s">
         <v>146</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="I6" s="45" t="s">
+      <c r="I6" s="36" t="s">
         <v>148</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="K6" s="40">
+      <c r="K6" s="31">
         <v>4500</v>
       </c>
-      <c r="L6" s="40">
+      <c r="L6" s="31">
         <v>810</v>
       </c>
-      <c r="M6" s="40">
+      <c r="M6" s="31">
         <v>5310</v>
       </c>
       <c r="N6" s="1" t="s">
@@ -2715,19 +3728,19 @@
       <c r="B7" s="1">
         <v>2</v>
       </c>
-      <c r="C7" s="42">
+      <c r="C7" s="33">
         <v>46044</v>
       </c>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="43" t="s">
+      <c r="E7" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="44" t="s">
+      <c r="F7" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="44" t="s">
+      <c r="G7" s="35" t="s">
         <v>151</v>
       </c>
       <c r="H7" s="1" t="s">
@@ -2739,13 +3752,13 @@
       <c r="J7" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="K7" s="40">
+      <c r="K7" s="31">
         <v>3200</v>
       </c>
-      <c r="L7" s="40">
+      <c r="L7" s="31">
         <v>576</v>
       </c>
-      <c r="M7" s="40">
+      <c r="M7" s="31">
         <v>3776</v>
       </c>
       <c r="N7" s="1" t="s">
@@ -2756,19 +3769,19 @@
       <c r="B8" s="1">
         <v>3</v>
       </c>
-      <c r="C8" s="42">
+      <c r="C8" s="33">
         <v>46058</v>
       </c>
-      <c r="D8" s="43" t="s">
+      <c r="D8" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="43" t="s">
+      <c r="E8" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="44" t="s">
+      <c r="F8" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="G8" s="44" t="s">
+      <c r="G8" s="35" t="s">
         <v>156</v>
       </c>
       <c r="H8" s="1" t="s">
@@ -2780,13 +3793,13 @@
       <c r="J8" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K8" s="40">
+      <c r="K8" s="31">
         <v>1800</v>
       </c>
-      <c r="L8" s="40">
+      <c r="L8" s="31">
         <v>324</v>
       </c>
-      <c r="M8" s="40">
+      <c r="M8" s="31">
         <v>2124</v>
       </c>
       <c r="N8" s="1" t="s">
@@ -2797,37 +3810,37 @@
       <c r="B9" s="1">
         <v>4</v>
       </c>
-      <c r="C9" s="42">
+      <c r="C9" s="33">
         <v>46071</v>
       </c>
-      <c r="D9" s="43" t="s">
+      <c r="D9" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="E9" s="43" t="s">
+      <c r="E9" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="F9" s="44" t="s">
+      <c r="F9" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="G9" s="44" t="s">
+      <c r="G9" s="35" t="s">
         <v>160</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="I9" s="45" t="s">
+      <c r="I9" s="36" t="s">
         <v>162</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K9" s="40">
+      <c r="K9" s="31">
         <v>12000</v>
       </c>
-      <c r="L9" s="40">
+      <c r="L9" s="31">
         <v>2160</v>
       </c>
-      <c r="M9" s="40">
+      <c r="M9" s="31">
         <v>14160</v>
       </c>
       <c r="N9" s="1" t="s">
@@ -2838,37 +3851,37 @@
       <c r="B10" s="1">
         <v>5</v>
       </c>
-      <c r="C10" s="42">
+      <c r="C10" s="33">
         <v>46084</v>
       </c>
-      <c r="D10" s="43" t="s">
+      <c r="D10" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="43" t="s">
+      <c r="E10" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="F10" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="G10" s="44" t="s">
+      <c r="G10" s="35" t="s">
         <v>151</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="I10" s="47" t="s">
+      <c r="I10" s="38" t="s">
         <v>165</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="K10" s="40">
+      <c r="K10" s="31">
         <v>20000</v>
       </c>
-      <c r="L10" s="40">
+      <c r="L10" s="31">
         <v>3600</v>
       </c>
-      <c r="M10" s="40">
+      <c r="M10" s="31">
         <v>23600</v>
       </c>
       <c r="N10" s="1" t="s">
@@ -2879,19 +3892,19 @@
       <c r="B11" s="1">
         <v>6</v>
       </c>
-      <c r="C11" s="42">
+      <c r="C11" s="33">
         <v>46100</v>
       </c>
-      <c r="D11" s="43" t="s">
+      <c r="D11" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="43" t="s">
+      <c r="E11" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="44" t="s">
+      <c r="F11" s="35" t="s">
         <v>59</v>
       </c>
-      <c r="G11" s="44" t="s">
+      <c r="G11" s="35" t="s">
         <v>58</v>
       </c>
       <c r="H11" s="1" t="s">
@@ -2903,13 +3916,13 @@
       <c r="J11" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="K11" s="40">
+      <c r="K11" s="31">
         <v>8500</v>
       </c>
-      <c r="L11" s="40">
+      <c r="L11" s="31">
         <v>1530</v>
       </c>
-      <c r="M11" s="40">
+      <c r="M11" s="31">
         <v>10030</v>
       </c>
       <c r="N11" s="1" t="s">
@@ -2920,19 +3933,19 @@
       <c r="B12" s="1">
         <v>7</v>
       </c>
-      <c r="C12" s="42">
+      <c r="C12" s="33">
         <v>46114</v>
       </c>
-      <c r="D12" s="43" t="s">
+      <c r="D12" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="E12" s="43" t="s">
+      <c r="E12" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="F12" s="44" t="s">
+      <c r="F12" s="35" t="s">
         <v>66</v>
       </c>
-      <c r="G12" s="44" t="s">
+      <c r="G12" s="35" t="s">
         <v>58</v>
       </c>
       <c r="H12" s="1" t="s">
@@ -2944,13 +3957,13 @@
       <c r="J12" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="K12" s="40">
+      <c r="K12" s="31">
         <v>9500</v>
       </c>
-      <c r="L12" s="40">
+      <c r="L12" s="31">
         <v>1710</v>
       </c>
-      <c r="M12" s="40">
+      <c r="M12" s="31">
         <v>11210</v>
       </c>
       <c r="N12" s="1" t="s">
@@ -2961,37 +3974,37 @@
       <c r="B13" s="1">
         <v>8</v>
       </c>
-      <c r="C13" s="42">
+      <c r="C13" s="33">
         <v>46127</v>
       </c>
-      <c r="D13" s="43" t="s">
+      <c r="D13" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="E13" s="43" t="s">
+      <c r="E13" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="F13" s="44" t="s">
+      <c r="F13" s="35" t="s">
         <v>73</v>
       </c>
-      <c r="G13" s="44" t="s">
+      <c r="G13" s="35" t="s">
         <v>72</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="I13" s="46" t="s">
+      <c r="I13" s="37" t="s">
         <v>174</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="K13" s="40">
+      <c r="K13" s="31">
         <v>15000</v>
       </c>
-      <c r="L13" s="40">
+      <c r="L13" s="31">
         <v>2700</v>
       </c>
-      <c r="M13" s="40">
+      <c r="M13" s="31">
         <v>17700</v>
       </c>
       <c r="N13" s="1" t="s">
@@ -3002,19 +4015,19 @@
       <c r="B14" s="1">
         <v>9</v>
       </c>
-      <c r="C14" s="42">
+      <c r="C14" s="33">
         <v>46148</v>
       </c>
-      <c r="D14" s="43" t="s">
+      <c r="D14" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="E14" s="43" t="s">
+      <c r="E14" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="F14" s="44" t="s">
+      <c r="F14" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="G14" s="44" t="s">
+      <c r="G14" s="35" t="s">
         <v>79</v>
       </c>
       <c r="H14" s="1" t="s">
@@ -3026,13 +4039,13 @@
       <c r="J14" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="K14" s="40">
+      <c r="K14" s="31">
         <v>22000</v>
       </c>
-      <c r="L14" s="40">
+      <c r="L14" s="31">
         <v>3960</v>
       </c>
-      <c r="M14" s="40">
+      <c r="M14" s="31">
         <v>25960</v>
       </c>
       <c r="N14" s="1" t="s">
@@ -3043,19 +4056,19 @@
       <c r="B15" s="1">
         <v>10</v>
       </c>
-      <c r="C15" s="42">
+      <c r="C15" s="33">
         <v>46162</v>
       </c>
-      <c r="D15" s="43" t="s">
+      <c r="D15" s="34" t="s">
         <v>81</v>
       </c>
-      <c r="E15" s="43" t="s">
+      <c r="E15" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="F15" s="44" t="s">
+      <c r="F15" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="G15" s="44" t="s">
+      <c r="G15" s="35" t="s">
         <v>85</v>
       </c>
       <c r="H15" s="1" t="s">
@@ -3067,13 +4080,13 @@
       <c r="J15" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="K15" s="40">
+      <c r="K15" s="31">
         <v>6000</v>
       </c>
-      <c r="L15" s="40">
+      <c r="L15" s="31">
         <v>1080</v>
       </c>
-      <c r="M15" s="40">
+      <c r="M15" s="31">
         <v>7080</v>
       </c>
       <c r="N15" s="1" t="s">
@@ -3084,37 +4097,37 @@
       <c r="B16" s="1">
         <v>11</v>
       </c>
-      <c r="C16" s="42">
+      <c r="C16" s="33">
         <v>46177</v>
       </c>
-      <c r="D16" s="43" t="s">
+      <c r="D16" s="34" t="s">
         <v>88</v>
       </c>
-      <c r="E16" s="43" t="s">
+      <c r="E16" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="F16" s="44" t="s">
+      <c r="F16" s="35" t="s">
         <v>92</v>
       </c>
-      <c r="G16" s="44" t="s">
+      <c r="G16" s="35" t="s">
         <v>85</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="I16" s="45" t="s">
+      <c r="I16" s="36" t="s">
         <v>183</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="K16" s="40">
+      <c r="K16" s="31">
         <v>45000</v>
       </c>
-      <c r="L16" s="40">
+      <c r="L16" s="31">
         <v>8100</v>
       </c>
-      <c r="M16" s="40">
+      <c r="M16" s="31">
         <v>53100</v>
       </c>
       <c r="N16" s="1" t="s">
@@ -3125,19 +4138,19 @@
       <c r="B17" s="1">
         <v>12</v>
       </c>
-      <c r="C17" s="42">
+      <c r="C17" s="33">
         <v>46191</v>
       </c>
-      <c r="D17" s="43" t="s">
+      <c r="D17" s="34" t="s">
         <v>93</v>
       </c>
-      <c r="E17" s="43" t="s">
+      <c r="E17" s="34" t="s">
         <v>96</v>
       </c>
-      <c r="F17" s="44" t="s">
+      <c r="F17" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="G17" s="44" t="s">
+      <c r="G17" s="35" t="s">
         <v>97</v>
       </c>
       <c r="H17" s="1" t="s">
@@ -3149,13 +4162,13 @@
       <c r="J17" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="K17" s="40">
+      <c r="K17" s="31">
         <v>18000</v>
       </c>
-      <c r="L17" s="40">
+      <c r="L17" s="31">
         <v>3240</v>
       </c>
-      <c r="M17" s="40">
+      <c r="M17" s="31">
         <v>21240</v>
       </c>
       <c r="N17" s="1" t="s">
@@ -3166,19 +4179,19 @@
       <c r="B18" s="1">
         <v>13</v>
       </c>
-      <c r="C18" s="42">
+      <c r="C18" s="33">
         <v>46210</v>
       </c>
-      <c r="D18" s="43" t="s">
+      <c r="D18" s="34" t="s">
         <v>100</v>
       </c>
-      <c r="E18" s="43" t="s">
+      <c r="E18" s="34" t="s">
         <v>189</v>
       </c>
-      <c r="F18" s="44" t="s">
+      <c r="F18" s="35" t="s">
         <v>106</v>
       </c>
-      <c r="G18" s="44" t="s">
+      <c r="G18" s="35" t="s">
         <v>105</v>
       </c>
       <c r="H18" s="1" t="s">
@@ -3190,13 +4203,13 @@
       <c r="J18" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="K18" s="40">
+      <c r="K18" s="31">
         <v>12000</v>
       </c>
-      <c r="L18" s="40">
+      <c r="L18" s="31">
         <v>2160</v>
       </c>
-      <c r="M18" s="40">
+      <c r="M18" s="31">
         <v>14160</v>
       </c>
       <c r="N18" s="1" t="s">
@@ -3207,19 +4220,19 @@
       <c r="B19" s="1">
         <v>14</v>
       </c>
-      <c r="C19" s="42">
+      <c r="C19" s="33">
         <v>46224</v>
       </c>
-      <c r="D19" s="43" t="s">
+      <c r="D19" s="34" t="s">
         <v>107</v>
       </c>
-      <c r="E19" s="43" t="s">
+      <c r="E19" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="F19" s="44" t="s">
+      <c r="F19" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="G19" s="44" t="s">
+      <c r="G19" s="35" t="s">
         <v>151</v>
       </c>
       <c r="H19" s="1" t="s">
@@ -3231,13 +4244,13 @@
       <c r="J19" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="K19" s="40">
+      <c r="K19" s="31">
         <v>7000</v>
       </c>
-      <c r="L19" s="40">
+      <c r="L19" s="31">
         <v>1260</v>
       </c>
-      <c r="M19" s="40">
+      <c r="M19" s="31">
         <v>8260</v>
       </c>
       <c r="N19" s="1" t="s">
@@ -3248,19 +4261,19 @@
       <c r="B20" s="1">
         <v>15</v>
       </c>
-      <c r="C20" s="42">
+      <c r="C20" s="33">
         <v>46239</v>
       </c>
-      <c r="D20" s="43" t="s">
+      <c r="D20" s="34" t="s">
         <v>112</v>
       </c>
-      <c r="E20" s="43" t="s">
+      <c r="E20" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="F20" s="44" t="s">
+      <c r="F20" s="35" t="s">
         <v>116</v>
       </c>
-      <c r="G20" s="44" t="s">
+      <c r="G20" s="35" t="s">
         <v>151</v>
       </c>
       <c r="H20" s="1" t="s">
@@ -3272,13 +4285,13 @@
       <c r="J20" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="K20" s="40">
+      <c r="K20" s="31">
         <v>1500</v>
       </c>
-      <c r="L20" s="40">
+      <c r="L20" s="31">
         <v>270</v>
       </c>
-      <c r="M20" s="40">
+      <c r="M20" s="31">
         <v>1770</v>
       </c>
       <c r="N20" s="1" t="s">
@@ -3289,19 +4302,19 @@
       <c r="B21" s="1">
         <v>16</v>
       </c>
-      <c r="C21" s="42">
+      <c r="C21" s="33">
         <v>46253</v>
       </c>
-      <c r="D21" s="43" t="s">
+      <c r="D21" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="E21" s="43" t="s">
+      <c r="E21" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="F21" s="44" t="s">
+      <c r="F21" s="35" t="s">
         <v>122</v>
       </c>
-      <c r="G21" s="44" t="s">
+      <c r="G21" s="35" t="s">
         <v>121</v>
       </c>
       <c r="H21" s="1" t="s">
@@ -3313,13 +4326,13 @@
       <c r="J21" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="K21" s="40">
+      <c r="K21" s="31">
         <v>5000</v>
       </c>
-      <c r="L21" s="40">
+      <c r="L21" s="31">
         <v>900</v>
       </c>
-      <c r="M21" s="40">
+      <c r="M21" s="31">
         <v>5900</v>
       </c>
       <c r="N21" s="1" t="s">
@@ -3330,37 +4343,37 @@
       <c r="B22" s="1">
         <v>17</v>
       </c>
-      <c r="C22" s="42">
+      <c r="C22" s="33">
         <v>46268</v>
       </c>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="34" t="s">
         <v>123</v>
       </c>
-      <c r="E22" s="43" t="s">
+      <c r="E22" s="34" t="s">
         <v>202</v>
       </c>
-      <c r="F22" s="44" t="s">
+      <c r="F22" s="35" t="s">
         <v>128</v>
       </c>
-      <c r="G22" s="44" t="s">
+      <c r="G22" s="35" t="s">
         <v>121</v>
       </c>
       <c r="H22" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="I22" s="45" t="s">
+      <c r="I22" s="36" t="s">
         <v>203</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="K22" s="40">
+      <c r="K22" s="31">
         <v>25000</v>
       </c>
-      <c r="L22" s="40">
+      <c r="L22" s="31">
         <v>4500</v>
       </c>
-      <c r="M22" s="40">
+      <c r="M22" s="31">
         <v>29500</v>
       </c>
       <c r="N22" s="1" t="s">
@@ -3371,19 +4384,19 @@
       <c r="B23" s="1">
         <v>18</v>
       </c>
-      <c r="C23" s="42">
+      <c r="C23" s="33">
         <v>46282</v>
       </c>
-      <c r="D23" s="43" t="s">
+      <c r="D23" s="34" t="s">
         <v>129</v>
       </c>
-      <c r="E23" s="43" t="s">
+      <c r="E23" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="F23" s="44" t="s">
+      <c r="F23" s="35" t="s">
         <v>134</v>
       </c>
-      <c r="G23" s="44" t="s">
+      <c r="G23" s="35" t="s">
         <v>133</v>
       </c>
       <c r="H23" s="1" t="s">
@@ -3395,13 +4408,13 @@
       <c r="J23" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="K23" s="40">
+      <c r="K23" s="31">
         <v>11000</v>
       </c>
-      <c r="L23" s="40">
+      <c r="L23" s="31">
         <v>1980</v>
       </c>
-      <c r="M23" s="40">
+      <c r="M23" s="31">
         <v>12980</v>
       </c>
       <c r="N23" s="1" t="s">
@@ -3414,4 +4427,984 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57F1CE08-004D-462B-9BB8-BFB59242CF94}">
+  <dimension ref="B1:P23"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" customWidth="1"/>
+    <col min="12" max="12" width="13.28515625" customWidth="1"/>
+    <col min="13" max="13" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:16">
+      <c r="B1" s="70" t="s">
+        <v>209</v>
+      </c>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+    </row>
+    <row r="2" spans="2:16">
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
+      <c r="M2" s="71"/>
+      <c r="N2" s="71"/>
+      <c r="O2" s="71"/>
+    </row>
+    <row r="3" spans="2:16">
+      <c r="B3" s="71"/>
+      <c r="C3" s="71"/>
+      <c r="D3" s="71"/>
+      <c r="E3" s="71"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71"/>
+      <c r="I3" s="71"/>
+      <c r="J3" s="71"/>
+      <c r="K3" s="71"/>
+      <c r="L3" s="71"/>
+      <c r="M3" s="71"/>
+      <c r="N3" s="71"/>
+      <c r="O3" s="71"/>
+    </row>
+    <row r="4" spans="2:16">
+      <c r="B4" s="67" t="s">
+        <v>210</v>
+      </c>
+      <c r="C4" s="68"/>
+      <c r="D4" s="68"/>
+      <c r="E4" s="68"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="67" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="68"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="69"/>
+      <c r="K4" s="67" t="s">
+        <v>212</v>
+      </c>
+      <c r="L4" s="68"/>
+      <c r="M4" s="68"/>
+      <c r="N4" s="68"/>
+      <c r="O4" s="68"/>
+      <c r="P4" s="51"/>
+    </row>
+    <row r="5" spans="2:16">
+      <c r="B5" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="F5" s="54" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="J5" s="54" t="s">
+        <v>219</v>
+      </c>
+      <c r="K5" s="15" t="s">
+        <v>220</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="N5" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="O5" s="54" t="s">
+        <v>145</v>
+      </c>
+      <c r="P5" s="52"/>
+    </row>
+    <row r="6" spans="2:16">
+      <c r="B6" s="16">
+        <v>1</v>
+      </c>
+      <c r="C6" s="64" t="s">
+        <v>223</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="F6" s="53" t="s">
+        <v>226</v>
+      </c>
+      <c r="G6" s="58" t="s">
+        <v>227</v>
+      </c>
+      <c r="H6" s="59">
+        <v>9876501234</v>
+      </c>
+      <c r="I6" s="59" t="s">
+        <v>228</v>
+      </c>
+      <c r="J6" s="60" t="s">
+        <v>229</v>
+      </c>
+      <c r="K6" s="16">
+        <v>30</v>
+      </c>
+      <c r="L6" s="1">
+        <v>75</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="N6" s="33">
+        <v>46027</v>
+      </c>
+      <c r="O6" s="53" t="s">
+        <v>231</v>
+      </c>
+      <c r="P6" s="52"/>
+    </row>
+    <row r="7" spans="2:16">
+      <c r="B7" s="16">
+        <v>2</v>
+      </c>
+      <c r="C7" s="64" t="s">
+        <v>232</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="F7" s="53" t="s">
+        <v>234</v>
+      </c>
+      <c r="G7" s="58" t="s">
+        <v>235</v>
+      </c>
+      <c r="H7" s="59">
+        <v>9876543210</v>
+      </c>
+      <c r="I7" s="59" t="s">
+        <v>236</v>
+      </c>
+      <c r="J7" s="60" t="s">
+        <v>229</v>
+      </c>
+      <c r="K7" s="16">
+        <v>25</v>
+      </c>
+      <c r="L7" s="1">
+        <v>60</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="N7" s="33">
+        <v>46032</v>
+      </c>
+      <c r="O7" s="53" t="s">
+        <v>238</v>
+      </c>
+      <c r="P7" s="52"/>
+    </row>
+    <row r="8" spans="2:16">
+      <c r="B8" s="16">
+        <v>3</v>
+      </c>
+      <c r="C8" s="64" t="s">
+        <v>239</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="F8" s="53" t="s">
+        <v>242</v>
+      </c>
+      <c r="G8" s="58" t="s">
+        <v>243</v>
+      </c>
+      <c r="H8" s="59">
+        <v>9011223344</v>
+      </c>
+      <c r="I8" s="59" t="s">
+        <v>244</v>
+      </c>
+      <c r="J8" s="60" t="s">
+        <v>229</v>
+      </c>
+      <c r="K8" s="16">
+        <v>20</v>
+      </c>
+      <c r="L8" s="1">
+        <v>45</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="N8" s="33">
+        <v>46037</v>
+      </c>
+      <c r="O8" s="53" t="s">
+        <v>246</v>
+      </c>
+      <c r="P8" s="52"/>
+    </row>
+    <row r="9" spans="2:16">
+      <c r="B9" s="16">
+        <v>4</v>
+      </c>
+      <c r="C9" s="64" t="s">
+        <v>247</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="F9" s="53" t="s">
+        <v>242</v>
+      </c>
+      <c r="G9" s="58" t="s">
+        <v>250</v>
+      </c>
+      <c r="H9" s="59">
+        <v>9870011223</v>
+      </c>
+      <c r="I9" s="59" t="s">
+        <v>251</v>
+      </c>
+      <c r="J9" s="60" t="s">
+        <v>252</v>
+      </c>
+      <c r="K9" s="16">
+        <v>15</v>
+      </c>
+      <c r="L9" s="1">
+        <v>28</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="N9" s="33">
+        <v>46042</v>
+      </c>
+      <c r="O9" s="53" t="s">
+        <v>254</v>
+      </c>
+      <c r="P9" s="52"/>
+    </row>
+    <row r="10" spans="2:16">
+      <c r="B10" s="16">
+        <v>5</v>
+      </c>
+      <c r="C10" s="64" t="s">
+        <v>255</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="F10" s="53" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="58" t="s">
+        <v>258</v>
+      </c>
+      <c r="H10" s="59">
+        <v>9012345678</v>
+      </c>
+      <c r="I10" s="59" t="s">
+        <v>259</v>
+      </c>
+      <c r="J10" s="60" t="s">
+        <v>252</v>
+      </c>
+      <c r="K10" s="16">
+        <v>15</v>
+      </c>
+      <c r="L10" s="1">
+        <v>40</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="N10" s="33">
+        <v>46047</v>
+      </c>
+      <c r="O10" s="53" t="s">
+        <v>261</v>
+      </c>
+      <c r="P10" s="52"/>
+    </row>
+    <row r="11" spans="2:16">
+      <c r="B11" s="16">
+        <v>6</v>
+      </c>
+      <c r="C11" s="64" t="s">
+        <v>262</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="F11" s="53" t="s">
+        <v>226</v>
+      </c>
+      <c r="G11" s="58" t="s">
+        <v>227</v>
+      </c>
+      <c r="H11" s="59">
+        <v>9876501234</v>
+      </c>
+      <c r="I11" s="59" t="s">
+        <v>228</v>
+      </c>
+      <c r="J11" s="60" t="s">
+        <v>264</v>
+      </c>
+      <c r="K11" s="16">
+        <v>40</v>
+      </c>
+      <c r="L11" s="1">
+        <v>85</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="N11" s="33">
+        <v>46054</v>
+      </c>
+      <c r="O11" s="53" t="s">
+        <v>266</v>
+      </c>
+      <c r="P11" s="52"/>
+    </row>
+    <row r="12" spans="2:16">
+      <c r="B12" s="16">
+        <v>7</v>
+      </c>
+      <c r="C12" s="64" t="s">
+        <v>267</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="F12" s="53" t="s">
+        <v>269</v>
+      </c>
+      <c r="G12" s="58" t="s">
+        <v>270</v>
+      </c>
+      <c r="H12" s="59">
+        <v>9123987654</v>
+      </c>
+      <c r="I12" s="59" t="s">
+        <v>271</v>
+      </c>
+      <c r="J12" s="60" t="s">
+        <v>229</v>
+      </c>
+      <c r="K12" s="16">
+        <v>20</v>
+      </c>
+      <c r="L12" s="1">
+        <v>52</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="N12" s="33">
+        <v>46058</v>
+      </c>
+      <c r="O12" s="53" t="s">
+        <v>273</v>
+      </c>
+      <c r="P12" s="52"/>
+    </row>
+    <row r="13" spans="2:16">
+      <c r="B13" s="16">
+        <v>8</v>
+      </c>
+      <c r="C13" s="64" t="s">
+        <v>274</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="F13" s="53" t="s">
+        <v>276</v>
+      </c>
+      <c r="G13" s="58" t="s">
+        <v>277</v>
+      </c>
+      <c r="H13" s="59">
+        <v>9988123456</v>
+      </c>
+      <c r="I13" s="59" t="s">
+        <v>278</v>
+      </c>
+      <c r="J13" s="60" t="s">
+        <v>229</v>
+      </c>
+      <c r="K13" s="16">
+        <v>15</v>
+      </c>
+      <c r="L13" s="1">
+        <v>48</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="N13" s="33">
+        <v>46063</v>
+      </c>
+      <c r="O13" s="53" t="s">
+        <v>280</v>
+      </c>
+      <c r="P13" s="52"/>
+    </row>
+    <row r="14" spans="2:16">
+      <c r="B14" s="16">
+        <v>9</v>
+      </c>
+      <c r="C14" s="64" t="s">
+        <v>281</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="F14" s="53" t="s">
+        <v>283</v>
+      </c>
+      <c r="G14" s="58" t="s">
+        <v>284</v>
+      </c>
+      <c r="H14" s="59">
+        <v>9345612789</v>
+      </c>
+      <c r="I14" s="59" t="s">
+        <v>285</v>
+      </c>
+      <c r="J14" s="60" t="s">
+        <v>252</v>
+      </c>
+      <c r="K14" s="16">
+        <v>25</v>
+      </c>
+      <c r="L14" s="1">
+        <v>60</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="N14" s="33">
+        <v>46068</v>
+      </c>
+      <c r="O14" s="53" t="s">
+        <v>287</v>
+      </c>
+      <c r="P14" s="52"/>
+    </row>
+    <row r="15" spans="2:16">
+      <c r="B15" s="16">
+        <v>10</v>
+      </c>
+      <c r="C15" s="64" t="s">
+        <v>288</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="F15" s="53" t="s">
+        <v>291</v>
+      </c>
+      <c r="G15" s="58" t="s">
+        <v>292</v>
+      </c>
+      <c r="H15" s="59">
+        <v>9098765432</v>
+      </c>
+      <c r="I15" s="59" t="s">
+        <v>293</v>
+      </c>
+      <c r="J15" s="60" t="s">
+        <v>252</v>
+      </c>
+      <c r="K15" s="16">
+        <v>10</v>
+      </c>
+      <c r="L15" s="1">
+        <v>25</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="N15" s="33">
+        <v>46073</v>
+      </c>
+      <c r="O15" s="53" t="s">
+        <v>254</v>
+      </c>
+      <c r="P15" s="52"/>
+    </row>
+    <row r="16" spans="2:16">
+      <c r="B16" s="16">
+        <v>11</v>
+      </c>
+      <c r="C16" s="64" t="s">
+        <v>295</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="F16" s="53" t="s">
+        <v>297</v>
+      </c>
+      <c r="G16" s="58" t="s">
+        <v>298</v>
+      </c>
+      <c r="H16" s="59">
+        <v>9012340000</v>
+      </c>
+      <c r="I16" s="59" t="s">
+        <v>299</v>
+      </c>
+      <c r="J16" s="60" t="s">
+        <v>252</v>
+      </c>
+      <c r="K16" s="16">
+        <v>20</v>
+      </c>
+      <c r="L16" s="1">
+        <v>35</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="N16" s="33">
+        <v>46078</v>
+      </c>
+      <c r="O16" s="53" t="s">
+        <v>254</v>
+      </c>
+      <c r="P16" s="52"/>
+    </row>
+    <row r="17" spans="2:16">
+      <c r="B17" s="16">
+        <v>12</v>
+      </c>
+      <c r="C17" s="64" t="s">
+        <v>301</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="F17" s="53" t="s">
+        <v>291</v>
+      </c>
+      <c r="G17" s="58" t="s">
+        <v>292</v>
+      </c>
+      <c r="H17" s="59">
+        <v>9098765432</v>
+      </c>
+      <c r="I17" s="59" t="s">
+        <v>293</v>
+      </c>
+      <c r="J17" s="60" t="s">
+        <v>252</v>
+      </c>
+      <c r="K17" s="16">
+        <v>15</v>
+      </c>
+      <c r="L17" s="1">
+        <v>33</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="N17" s="33">
+        <v>46082</v>
+      </c>
+      <c r="O17" s="53" t="s">
+        <v>254</v>
+      </c>
+      <c r="P17" s="52"/>
+    </row>
+    <row r="18" spans="2:16">
+      <c r="B18" s="16">
+        <v>13</v>
+      </c>
+      <c r="C18" s="64" t="s">
+        <v>304</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="F18" s="53" t="s">
+        <v>242</v>
+      </c>
+      <c r="G18" s="58" t="s">
+        <v>250</v>
+      </c>
+      <c r="H18" s="59">
+        <v>9870011223</v>
+      </c>
+      <c r="I18" s="59" t="s">
+        <v>251</v>
+      </c>
+      <c r="J18" s="60" t="s">
+        <v>306</v>
+      </c>
+      <c r="K18" s="16">
+        <v>10</v>
+      </c>
+      <c r="L18" s="1">
+        <v>22</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="N18" s="33">
+        <v>46086</v>
+      </c>
+      <c r="O18" s="53" t="s">
+        <v>308</v>
+      </c>
+      <c r="P18" s="52"/>
+    </row>
+    <row r="19" spans="2:16">
+      <c r="B19" s="16">
+        <v>14</v>
+      </c>
+      <c r="C19" s="64" t="s">
+        <v>309</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="F19" s="53" t="s">
+        <v>311</v>
+      </c>
+      <c r="G19" s="58" t="s">
+        <v>312</v>
+      </c>
+      <c r="H19" s="59">
+        <v>9345678901</v>
+      </c>
+      <c r="I19" s="59" t="s">
+        <v>313</v>
+      </c>
+      <c r="J19" s="60" t="s">
+        <v>306</v>
+      </c>
+      <c r="K19" s="16">
+        <v>30</v>
+      </c>
+      <c r="L19" s="1">
+        <v>75</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="N19" s="33">
+        <v>46091</v>
+      </c>
+      <c r="O19" s="53" t="s">
+        <v>314</v>
+      </c>
+      <c r="P19" s="52"/>
+    </row>
+    <row r="20" spans="2:16">
+      <c r="B20" s="16">
+        <v>15</v>
+      </c>
+      <c r="C20" s="64" t="s">
+        <v>315</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="F20" s="53" t="s">
+        <v>283</v>
+      </c>
+      <c r="G20" s="58" t="s">
+        <v>284</v>
+      </c>
+      <c r="H20" s="59">
+        <v>9345612789</v>
+      </c>
+      <c r="I20" s="59" t="s">
+        <v>285</v>
+      </c>
+      <c r="J20" s="60" t="s">
+        <v>306</v>
+      </c>
+      <c r="K20" s="16">
+        <v>20</v>
+      </c>
+      <c r="L20" s="1">
+        <v>40</v>
+      </c>
+      <c r="M20" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="N20" s="33">
+        <v>46096</v>
+      </c>
+      <c r="O20" s="53" t="s">
+        <v>317</v>
+      </c>
+      <c r="P20" s="52"/>
+    </row>
+    <row r="21" spans="2:16">
+      <c r="B21" s="16">
+        <v>16</v>
+      </c>
+      <c r="C21" s="64" t="s">
+        <v>318</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="F21" s="53" t="s">
+        <v>276</v>
+      </c>
+      <c r="G21" s="58" t="s">
+        <v>277</v>
+      </c>
+      <c r="H21" s="59">
+        <v>9988123456</v>
+      </c>
+      <c r="I21" s="59" t="s">
+        <v>278</v>
+      </c>
+      <c r="J21" s="60" t="s">
+        <v>229</v>
+      </c>
+      <c r="K21" s="16">
+        <v>20</v>
+      </c>
+      <c r="L21" s="1">
+        <v>35</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="N21" s="33">
+        <v>46101</v>
+      </c>
+      <c r="O21" s="53" t="s">
+        <v>321</v>
+      </c>
+      <c r="P21" s="52"/>
+    </row>
+    <row r="22" spans="2:16">
+      <c r="B22" s="16">
+        <v>17</v>
+      </c>
+      <c r="C22" s="64" t="s">
+        <v>322</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="F22" s="53" t="s">
+        <v>311</v>
+      </c>
+      <c r="G22" s="58" t="s">
+        <v>324</v>
+      </c>
+      <c r="H22" s="59">
+        <v>9123450000</v>
+      </c>
+      <c r="I22" s="59" t="s">
+        <v>325</v>
+      </c>
+      <c r="J22" s="60" t="s">
+        <v>306</v>
+      </c>
+      <c r="K22" s="16">
+        <v>25</v>
+      </c>
+      <c r="L22" s="1">
+        <v>50</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="N22" s="33">
+        <v>46106</v>
+      </c>
+      <c r="O22" s="53" t="s">
+        <v>327</v>
+      </c>
+      <c r="P22" s="52"/>
+    </row>
+    <row r="23" spans="2:16">
+      <c r="B23" s="55">
+        <v>18</v>
+      </c>
+      <c r="C23" s="65" t="s">
+        <v>328</v>
+      </c>
+      <c r="D23" s="56" t="s">
+        <v>329</v>
+      </c>
+      <c r="E23" s="56" t="s">
+        <v>330</v>
+      </c>
+      <c r="F23" s="57" t="s">
+        <v>331</v>
+      </c>
+      <c r="G23" s="61" t="s">
+        <v>312</v>
+      </c>
+      <c r="H23" s="62">
+        <v>9011223344</v>
+      </c>
+      <c r="I23" s="62" t="s">
+        <v>332</v>
+      </c>
+      <c r="J23" s="63" t="s">
+        <v>252</v>
+      </c>
+      <c r="K23" s="55">
+        <v>30</v>
+      </c>
+      <c r="L23" s="56">
+        <v>60</v>
+      </c>
+      <c r="M23" s="56" t="s">
+        <v>333</v>
+      </c>
+      <c r="N23" s="66">
+        <v>46111</v>
+      </c>
+      <c r="O23" s="57" t="s">
+        <v>254</v>
+      </c>
+      <c r="P23" s="52"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B1:O3"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="K4:O4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="L6:L23">
+    <cfRule type="cellIs" dxfId="30" priority="4" operator="lessThan">
+      <formula>$K$6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K6">
+    <cfRule type="cellIs" dxfId="29" priority="2" operator="lessThan">
+      <formula>$K$6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L6:L23">
+    <cfRule type="cellIs" dxfId="28" priority="1" operator="greaterThan">
+      <formula>$K$6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="3">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>